<commit_message>
Fill HSK1_parts_of_speech_2(51-100).xlsx with parts of speech
</commit_message>
<xml_diff>
--- a/HSK1_parts_of_speech_2(51-100).xlsx
+++ b/HSK1_parts_of_speech_2(51-100).xlsx
@@ -601,6 +601,11 @@
           <t>надевать, носить</t>
         </is>
       </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>надевать, носить (穿 衣服)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -627,6 +632,16 @@
           <t>кровать</t>
         </is>
       </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>кровать</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>для предметов постельного обихода: 一床被子 — одно одеяло</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -653,6 +668,11 @@
           <t>раз (счётное слово для событий, действий)</t>
         </is>
       </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>раз (счётное слово для событий и действий: 三次 — три раза)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -679,6 +699,16 @@
           <t>из, с</t>
         </is>
       </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>с самого начала, всегда (从不说 — никогда не говорит с самого начала)</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>из, с, от (место: 从中国来 — из Китая)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -705,6 +735,21 @@
           <t>ошибка; ошибочный</t>
         </is>
       </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>ошибка (出一个错 — сделать одну ошибку)</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>ошибаться, промахиваться (写错了字 — ошибся в написании)</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>ошибочный, неверный (错了 — неправильно)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -731,6 +776,11 @@
           <t>бить, ударять</t>
         </is>
       </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>бить, ударять; играть (в спорт); звонить; брать (такси) — многофункциональный глагол</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -762,6 +812,11 @@
           <t>да</t>
         </is>
       </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>словосочетание (глагол + существительное: 打 + 车), устойчивое выражение «взять такси»</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -793,6 +848,11 @@
           <t>да</t>
         </is>
       </c>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t>словосочетание (глагол + существительное: 打 + 电话), устойчивое выражение «звонить по телефону»</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -824,6 +884,11 @@
           <t>да</t>
         </is>
       </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>открыть; включить (离合词: 打开门 / 把门打开)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -855,6 +920,11 @@
           <t>да</t>
         </is>
       </c>
+      <c r="X11" t="inlineStr">
+        <is>
+          <t>словосочетание (глагол + существительное: 打 + 球), «играть в мяч»</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -881,6 +951,16 @@
           <t>большой</t>
         </is>
       </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>большой, крупный; взрослый</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>сильно, очень (声音大一点 — погромче)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -907,6 +987,11 @@
           <t>университет</t>
         </is>
       </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>университет, вуз</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -933,6 +1018,11 @@
           <t>студент</t>
         </is>
       </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>студент (вуза)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -959,6 +1049,16 @@
           <t>доходить (до)</t>
         </is>
       </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>доходить, прибывать (到机场 — прибыть в аэропорт)</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>до (时间/地点: 三点到 — до трёх часов)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -985,6 +1085,11 @@
           <t>получить, добиться</t>
         </is>
       </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>получить, добиться (离合词: 得到帮助)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1011,6 +1116,16 @@
           <t>частица для образования обстоятельств</t>
         </is>
       </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>частица обстоятельства: связывает наречие с глаголом (慢慢地走 — идти медленно)</t>
+        </is>
+      </c>
+      <c r="Y17" t="inlineStr">
+        <is>
+          <t>Самостоятельно не употребляется (служебная частица)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1037,6 +1152,16 @@
           <t>определительная частица</t>
         </is>
       </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>определительная частица: связывает определение с существительным (我的书 — моя книга)</t>
+        </is>
+      </c>
+      <c r="Y18" t="inlineStr">
+        <is>
+          <t>Самостоятельно не употребляется (служебная частица)</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1063,6 +1188,16 @@
           <t>ждать</t>
         </is>
       </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>ждать (等人 — ждать человека)</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>и так далее, -и проч. (桌子、椅子等 — столы, стулья и т.д.)</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1089,6 +1224,11 @@
           <t>земля</t>
         </is>
       </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>земля, пол, почва (在地上 — на земле)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1115,6 +1255,11 @@
           <t>пункт (географический)</t>
         </is>
       </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>место, точка (географическая)</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1141,6 +1286,11 @@
           <t>местный; местоположение</t>
         </is>
       </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>место, местность, регион</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1167,6 +1317,11 @@
           <t>на земле</t>
         </is>
       </c>
+      <c r="X23" t="inlineStr">
+        <is>
+          <t>словосочетание (существительное + локатив: 地 + 上), «на земле / на полу»</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1193,6 +1348,11 @@
           <t>карта</t>
         </is>
       </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>карта (地理)</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1224,6 +1384,11 @@
           <t>младший брат</t>
         </is>
       </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>младший брат</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1255,6 +1420,16 @@
           <t>префикс для образования порядковых числительных</t>
         </is>
       </c>
+      <c r="W26" t="inlineStr">
+        <is>
+          <t>приставка для порядковых числительных: 第一 — первый, 第三 — третий</t>
+        </is>
+      </c>
+      <c r="Y26" t="inlineStr">
+        <is>
+          <t>Самостоятельно не употребляется (приставка, только с числительным)</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1281,6 +1456,16 @@
           <t>точка</t>
         </is>
       </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>точка; час (о времени: 三点 — три часа); пункт, очко</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>для очков/баллов и процентов: 高十点 (на 10 баллов выше), 下降两点 (упал на 2 пункта)</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1312,6 +1497,11 @@
           <t>нет</t>
         </is>
       </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>электричество, электрический ток (来电 — подать электричество)</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1343,6 +1533,11 @@
           <t>да</t>
         </is>
       </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>телефон</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1374,6 +1569,11 @@
           <t>да</t>
         </is>
       </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>компьютер</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1405,6 +1605,11 @@
           <t>да</t>
         </is>
       </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>телевидение (看电視 — смотреть телевизор)</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -1436,6 +1641,11 @@
           <t>да</t>
         </is>
       </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>телевизор (прибор)</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1467,6 +1677,11 @@
           <t>да</t>
         </is>
       </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>фильм, кино</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -1498,6 +1713,11 @@
           <t>да</t>
         </is>
       </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>кинотеатр</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1524,6 +1744,11 @@
           <t>восток</t>
         </is>
       </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>восток (方向: 东边, 东方)</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -1550,6 +1775,11 @@
           <t>сторона, восток</t>
         </is>
       </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>восточная сторона, восток</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -1576,6 +1806,11 @@
           <t>вещь</t>
         </is>
       </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>вещь, предмет (买东西 — покупать вещи)</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -1602,6 +1837,11 @@
           <t>двигаться</t>
         </is>
       </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>двигаться, шевелиться; волновать (心动 — сердце ёкнуло)</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -1628,6 +1868,11 @@
           <t>движение</t>
         </is>
       </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>движение, действие (动作快一点 — быстрее)</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -1654,6 +1899,11 @@
           <t>все</t>
         </is>
       </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>все, оба, целиком (我们都去 — мы все идём)</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -1680,6 +1930,11 @@
           <t>читать</t>
         </is>
       </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>читать, читать вслух; изучать (读书 — учиться)</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -1706,6 +1961,11 @@
           <t>учиться; читать</t>
         </is>
       </c>
+      <c r="X42" t="inlineStr">
+        <is>
+          <t>словосочетание (глагол + существительное: 读 + 书), «учиться; читать книги»</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -1732,6 +1992,26 @@
           <t>верный, правильный</t>
         </is>
       </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>пара; спаренное (一对 — одна пара)</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>верный, правильный (说对了 — сказал верно)</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>для пар: 一对夫妻 — супружеская чета</t>
+        </is>
+      </c>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>по отношению к, кому-л. (对我很好 — ко мне добр)</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -1758,6 +2038,11 @@
           <t>Извините.</t>
         </is>
       </c>
+      <c r="U44" t="inlineStr">
+        <is>
+          <t>извините! (устойчивое формула вежливости 对不起)</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -1784,6 +2069,21 @@
           <t>много</t>
         </is>
       </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>иметь столько, превышать (多三个人 — на троих больше)</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>многочисленный, большой по количеству (人很多 — людей много)</t>
+        </is>
+      </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>как много!, сколько же (多好! — как хорошо!)</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -1810,6 +2110,11 @@
           <t>сколько</t>
         </is>
       </c>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>сколько? (疑问代词: 多少钱? — сколько стоит?)</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -1836,6 +2141,16 @@
           <t>голодный</t>
         </is>
       </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>голодать (饿了一天 — голодал день)</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>голодный (我很饿 — я очень голоден)</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -1867,6 +2182,11 @@
           <t>да</t>
         </is>
       </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>сын</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -1893,6 +2213,11 @@
           <t>два</t>
         </is>
       </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>два (二两 — 2 лян; 第二 — второй; перед счётными словами обычно 两, а не 二)</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -1919,6 +2244,11 @@
           <t>рис; еда</t>
         </is>
       </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>рис (готовый к еде); еда, приём пищи (吃饭 — есть)</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -1943,6 +2273,11 @@
       <c r="I51" t="inlineStr">
         <is>
           <t>ресторан</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>ресторан, столовая, гостиница с рестораном</t>
         </is>
       </c>
     </row>

</xml_diff>